<commit_message>
Podpora pro povinné vzorce a dvojitý vstup (Úkol 5)
- Grader nyní načítá soubor dvakrát: jednou pro detekci vzorců (=...),
  jednou pro porovnání vypočtených hodnot
- Úkoly 2–6: student musí zadat vzorec — samotné číslo nestačí
- Úkol 1: zůstává bez požadavku na vzorec (text/čísla)
- Úkol 5: kontroluje oba sloupce D i E (oba musí být vzorce)
- Aktualizován klíč 03_Uvod_HZD.xlsx na novou verzi cvičení

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/answer_keys/03_Uvod_HZD.xlsx
+++ b/data/answer_keys/03_Uvod_HZD.xlsx
@@ -5,16 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgvsetin-my.sharepoint.com/personal/filip_senkerik_mgvsetin_cz/Documents/Přípravy/1 ročník + kvinta/27 Týden - Hromadné zpracování dat - Všech 10 příprav/01) Úvod do hromadného zpracování dat/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip.senkerik\Desktop\Aplikace pro opravu excel souborů\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="11_6A5CE4D4721292626CCCBF66E287EE4BA65FCFD4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7920A535-5BF3-4E77-930A-C70DA8F511EB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849254C3-0DFF-49DA-A848-8E74E2691AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pokyny" sheetId="1" r:id="rId1"/>
-    <sheet name="Klíč" sheetId="2" r:id="rId2"/>
+    <sheet name="Klíč" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="Úkol 1" sheetId="3" r:id="rId3"/>
     <sheet name="Úkol 2" sheetId="4" r:id="rId4"/>
     <sheet name="Úkol 3" sheetId="5" r:id="rId5"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="213">
   <si>
     <t>Hromadné zpracování dat – Cvičení (1. hodina)</t>
   </si>
@@ -453,6 +453,9 @@
     <t>🌟  Bonus:</t>
   </si>
   <si>
+    <t>Změň cenu paliva u Octavie na 45 Kč/l. Co se stalo s cenou paliva za cestu?</t>
+  </si>
+  <si>
     <t>Tvoje pozorování:</t>
   </si>
   <si>
@@ -688,12 +691,6 @@
   </si>
   <si>
     <t>Který z těchto závodníků by byl podle tebe nejlepší ve víceboji a proč?</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
-  <si>
-    <t>Změň cenu paliva u Octavie na 45 Kč/l. Co se stalo s cenou paliva za cestu? Poté nezapomeň změnit nazpět 38 Kč/l (kvůli bodům v úkolu)</t>
   </si>
 </sst>
 </file>
@@ -1337,7 +1334,7 @@
     <col min="5" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="26" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
@@ -1348,7 +1345,7 @@
       <c r="G2" s="12"/>
       <c r="H2" s="12"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
@@ -1359,7 +1356,7 @@
       <c r="G3" s="11"/>
       <c r="H3" s="11"/>
     </row>
-    <row r="5" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="13" t="s">
         <v>2</v>
       </c>
@@ -1368,7 +1365,7 @@
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
     </row>
-    <row r="6" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="13" t="s">
         <v>3</v>
       </c>
@@ -1377,12 +1374,12 @@
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
     </row>
-    <row r="8" spans="2:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="14" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="15" t="s">
         <v>5</v>
       </c>
@@ -1395,7 +1392,7 @@
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
     </row>
-    <row r="11" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="15" t="s">
         <v>7</v>
       </c>
@@ -1408,7 +1405,7 @@
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
-    <row r="12" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="15" t="s">
         <v>9</v>
       </c>
@@ -1421,7 +1418,7 @@
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
-    <row r="13" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="15" t="s">
         <v>11</v>
       </c>
@@ -1434,7 +1431,7 @@
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
     </row>
-    <row r="14" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="15" t="s">
         <v>13</v>
       </c>
@@ -1447,7 +1444,7 @@
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
-    <row r="15" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="15" t="s">
         <v>15</v>
       </c>
@@ -1460,12 +1457,12 @@
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
     </row>
-    <row r="17" spans="2:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B17" s="14" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="16" t="s">
         <v>18</v>
       </c>
@@ -1480,7 +1477,7 @@
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="16" t="s">
         <v>21</v>
       </c>
@@ -1495,7 +1492,7 @@
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="16" t="s">
         <v>24</v>
       </c>
@@ -1510,7 +1507,7 @@
       <c r="G21" s="9"/>
       <c r="H21" s="9"/>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="16" t="s">
         <v>27</v>
       </c>
@@ -1525,7 +1522,7 @@
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="16" t="s">
         <v>30</v>
       </c>
@@ -1540,7 +1537,7 @@
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="16" t="s">
         <v>33</v>
       </c>
@@ -1555,7 +1552,7 @@
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
     </row>
-    <row r="27" spans="2:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B27" s="8" t="s">
         <v>36</v>
       </c>
@@ -1563,7 +1560,7 @@
       <c r="D27" s="8"/>
       <c r="E27" s="7" t="str">
         <f>SUM('Úkol 1'!AB1,'Úkol 2'!AB1,'Úkol 3'!AB1,'Úkol 4'!AB1,'Úkol 5'!AB1,'Úkol 6'!AB1) &amp; " / " &amp; SUM('Úkol 1'!AB2,'Úkol 2'!AB2,'Úkol 3'!AB2,'Úkol 4'!AB2,'Úkol 5'!AB2,'Úkol 6'!AB2)</f>
-        <v>56 / 56</v>
+        <v>17 / 56</v>
       </c>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
@@ -1600,287 +1597,287 @@
   <dimension ref="A1:A107"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>432</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>563</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>391</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>800</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>1024</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>455</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>169</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>525600</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>300</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>406</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>29.25</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>16.64</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>1111.5</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43">
-        <v>1719.12</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+        <v>1718.16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>260</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>6.5</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>2.1320000000000001</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60">
-        <v>21610</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+        <v>22610</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>10950</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>6040</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63">
-        <v>18910</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+        <v>22660</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64">
-        <v>19690</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+        <v>16940</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>5760</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>6100</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>2840</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>25.43</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>32</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>18</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>25.57</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>32</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>28</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>30.75</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>12</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>187</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>11.987500000000001</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>11.5</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>7.1</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>13.074999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>0.17</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>2343</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>281.67</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>8</v>
       </c>
@@ -1897,20 +1894,20 @@
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" customWidth="1"/>
+    <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AB1" s="19">
         <f>COUNTIF(H17:H26,"✓")</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="2:28" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="6" t="s">
         <v>43</v>
       </c>
@@ -1924,7 +1921,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>44</v>
       </c>
@@ -1935,7 +1932,7 @@
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
     </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="9" t="s">
         <v>45</v>
       </c>
@@ -1946,7 +1943,7 @@
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="9" t="s">
         <v>46</v>
       </c>
@@ -1957,7 +1954,7 @@
       <c r="G6" s="9"/>
       <c r="H6" s="9"/>
     </row>
-    <row r="8" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20" t="s">
         <v>47</v>
       </c>
@@ -1974,7 +1971,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="21" t="s">
         <v>52</v>
       </c>
@@ -1992,7 +1989,7 @@
         <v>18.333333333333332</v>
       </c>
     </row>
-    <row r="10" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="21" t="s">
         <v>53</v>
       </c>
@@ -2010,7 +2007,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="21" t="s">
         <v>54</v>
       </c>
@@ -2028,7 +2025,7 @@
         <v>17.666666666666668</v>
       </c>
     </row>
-    <row r="12" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="21" t="s">
         <v>38</v>
       </c>
@@ -2046,7 +2043,7 @@
         <v>22.333333333333332</v>
       </c>
     </row>
-    <row r="13" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="21" t="s">
         <v>55</v>
       </c>
@@ -2064,7 +2061,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="21" t="s">
         <v>39</v>
       </c>
@@ -2082,12 +2079,12 @@
         <v>17.666666666666668</v>
       </c>
     </row>
-    <row r="16" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="24" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="25" t="s">
         <v>57</v>
       </c>
@@ -2098,7 +2095,6 @@
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="26">
-        <f>C10</f>
         <v>25</v>
       </c>
       <c r="H17" s="27" t="str">
@@ -2106,7 +2102,7 @@
         <v>✓</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="25" t="s">
         <v>59</v>
       </c>
@@ -2117,7 +2113,6 @@
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
       <c r="G18" s="26">
-        <f>E11</f>
         <v>20</v>
       </c>
       <c r="H18" s="27" t="str">
@@ -2125,7 +2120,7 @@
         <v>✓</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="25" t="s">
         <v>61</v>
       </c>
@@ -2135,16 +2130,13 @@
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
-      <c r="G19" s="26" t="str">
-        <f>B12</f>
-        <v>Dana</v>
-      </c>
+      <c r="G19" s="26"/>
       <c r="H19" s="27" t="str">
         <f>IF(TRIM(LOWER(G19))="","",IF(TRIM(LOWER(G19))=TRIM(LOWER(Klíč!A4)),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="25" t="s">
         <v>63</v>
       </c>
@@ -2154,15 +2146,13 @@
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
-      <c r="G20" s="26">
-        <v>21</v>
-      </c>
+      <c r="G20" s="26"/>
       <c r="H20" s="27" t="str">
         <f>IF(G20="","",IF(G20=Klíč!A5,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="25" t="s">
         <v>65</v>
       </c>
@@ -2172,15 +2162,13 @@
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
-      <c r="G21" s="26" t="s">
-        <v>39</v>
-      </c>
+      <c r="G21" s="26"/>
       <c r="H21" s="27" t="str">
         <f>IF(TRIM(LOWER(G21))="","",IF(TRIM(LOWER(G21))=TRIM(LOWER(Klíč!A6)),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="25" t="s">
         <v>67</v>
       </c>
@@ -2190,15 +2178,13 @@
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
-      <c r="G22" s="26">
-        <v>18</v>
-      </c>
+      <c r="G22" s="26"/>
       <c r="H22" s="27" t="str">
         <f>IF(G22="","",IF(G22=Klíč!A7,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="23" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="25" t="s">
         <v>69</v>
       </c>
@@ -2208,15 +2194,13 @@
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
-      <c r="G23" s="26" t="s">
-        <v>40</v>
-      </c>
+      <c r="G23" s="26"/>
       <c r="H23" s="27" t="str">
         <f>IF(TRIM(LOWER(G23))="","",IF(TRIM(LOWER(G23))=TRIM(LOWER(Klíč!A8)),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="25" t="s">
         <v>71</v>
       </c>
@@ -2226,15 +2210,13 @@
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
-      <c r="G24" s="26" t="s">
-        <v>41</v>
-      </c>
+      <c r="G24" s="26"/>
       <c r="H24" s="27" t="str">
         <f>IF(TRIM(LOWER(G24))="","",IF(TRIM(LOWER(G24))=TRIM(LOWER(Klíč!A9)),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="25" t="s">
         <v>73</v>
       </c>
@@ -2244,15 +2226,13 @@
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
-      <c r="G25" s="26">
-        <v>13</v>
-      </c>
+      <c r="G25" s="26"/>
       <c r="H25" s="27" t="str">
         <f>IF(G25="","",IF(G25=Klíč!A10,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="25" t="s">
         <v>75</v>
       </c>
@@ -2262,15 +2242,13 @@
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
-      <c r="G26" s="26" t="s">
-        <v>212</v>
-      </c>
+      <c r="G26" s="26"/>
       <c r="H26" s="27" t="str">
         <f>IF(TRIM(LOWER(G26))="","",IF(TRIM(LOWER(G26))=TRIM(LOWER(Klíč!A11)),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="28" spans="2:8" ht="18.5" x14ac:dyDescent="0.45">
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B28" s="8" t="s">
         <v>77</v>
       </c>
@@ -2279,7 +2257,7 @@
       <c r="E28" s="8"/>
       <c r="F28" s="7" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>10 / 10  bodů</v>
+        <v>2 / 10  bodů</v>
       </c>
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
@@ -2328,13 +2306,13 @@
     <col min="5" max="5" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AB1" s="19">
         <f>COUNTIF(E9:E20,"✓")</f>
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="2:28" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="6" t="s">
         <v>78</v>
       </c>
@@ -2347,7 +2325,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>44</v>
       </c>
@@ -2357,7 +2335,7 @@
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
     </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="9" t="s">
         <v>79</v>
       </c>
@@ -2367,7 +2345,7 @@
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="4" t="s">
         <v>80</v>
       </c>
@@ -2377,7 +2355,7 @@
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="8" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20" t="s">
         <v>81</v>
       </c>
@@ -2388,7 +2366,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="28" t="s">
         <v>84</v>
       </c>
@@ -2400,11 +2378,11 @@
         <v>432</v>
       </c>
       <c r="E9" s="27" t="str">
-        <f>IF(D9="","",IF(D9=Klíč!A20,"✓","✗"))</f>
+        <f>IF(D9="","",IF(NOT(_xlfn.ISFORMULA(D9)),"✗",IF(D9=Klíč!A20,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="10" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="28" t="s">
         <v>86</v>
       </c>
@@ -2412,14 +2390,15 @@
         <v>87</v>
       </c>
       <c r="D10" s="26">
+        <f>1000-437</f>
         <v>563</v>
       </c>
       <c r="E10" s="27" t="str">
-        <f>IF(D10="","",IF(D10=Klíč!A21,"✓","✗"))</f>
+        <f>IF(D10="","",IF(NOT(_xlfn.ISFORMULA(D10)),"✗",IF(D10=Klíč!A21,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="11" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="28" t="s">
         <v>88</v>
       </c>
@@ -2431,11 +2410,11 @@
         <v>391</v>
       </c>
       <c r="E11" s="27" t="str">
-        <f>IF(D11="","",IF(D11=Klíč!A22,"✓","✗"))</f>
+        <f>IF(D11="","",IF(NOT(_xlfn.ISFORMULA(D11)),"✗",IF(D11=Klíč!A22,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="12" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="28" t="s">
         <v>90</v>
       </c>
@@ -2447,11 +2426,11 @@
         <v>64</v>
       </c>
       <c r="E12" s="27" t="str">
-        <f>IF(D12="","",IF(D12=Klíč!A23,"✓","✗"))</f>
+        <f>IF(D12="","",IF(NOT(_xlfn.ISFORMULA(D12)),"✗",IF(D12=Klíč!A23,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="13" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="28" t="s">
         <v>92</v>
       </c>
@@ -2463,11 +2442,11 @@
         <v>800</v>
       </c>
       <c r="E13" s="27" t="str">
-        <f>IF(D13="","",IF(D13=Klíč!A24,"✓","✗"))</f>
+        <f>IF(D13="","",IF(NOT(_xlfn.ISFORMULA(D13)),"✗",IF(D13=Klíč!A24,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="14" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="28" t="s">
         <v>94</v>
       </c>
@@ -2479,11 +2458,11 @@
         <v>1024</v>
       </c>
       <c r="E14" s="27" t="str">
-        <f>IF(D14="","",IF(D14=Klíč!A25,"✓","✗"))</f>
+        <f>IF(D14="","",IF(NOT(_xlfn.ISFORMULA(D14)),"✗",IF(D14=Klíč!A25,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="15" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="28" t="s">
         <v>96</v>
       </c>
@@ -2491,15 +2470,15 @@
         <v>97</v>
       </c>
       <c r="D15" s="26">
-        <f>(250 - 50) / (2 + 8)</f>
+        <f>(250-50)/(2+8)</f>
         <v>20</v>
       </c>
       <c r="E15" s="27" t="str">
-        <f>IF(D15="","",IF(D15=Klíč!A26,"✓","✗"))</f>
+        <f>IF(D15="","",IF(NOT(_xlfn.ISFORMULA(D15)),"✗",IF(D15=Klíč!A26,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="16" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="28" t="s">
         <v>98</v>
       </c>
@@ -2507,15 +2486,15 @@
         <v>99</v>
       </c>
       <c r="D16" s="26">
-        <f>(7*60)+35</f>
+        <f>7*60+35</f>
         <v>455</v>
       </c>
       <c r="E16" s="27" t="str">
-        <f>IF(D16="","",IF(D16=Klíč!A27,"✓","✗"))</f>
+        <f>IF(D16="","",IF(NOT(_xlfn.ISFORMULA(D16)),"✗",IF(D16=Klíč!A27,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="28" t="s">
         <v>100</v>
       </c>
@@ -2527,11 +2506,11 @@
         <v>169</v>
       </c>
       <c r="E17" s="27" t="str">
-        <f>IF(D17="","",IF(D17=Klíč!A28,"✓","✗"))</f>
+        <f>IF(D17="","",IF(NOT(_xlfn.ISFORMULA(D17)),"✗",IF(D17=Klíč!A28,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="28" t="s">
         <v>102</v>
       </c>
@@ -2543,11 +2522,11 @@
         <v>525600</v>
       </c>
       <c r="E18" s="27" t="str">
-        <f>IF(D18="","",IF(D18=Klíč!A29,"✓","✗"))</f>
+        <f>IF(D18="","",IF(NOT(_xlfn.ISFORMULA(D18)),"✗",IF(D18=Klíč!A29,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="19" spans="2:5" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="28" t="s">
         <v>104</v>
       </c>
@@ -2559,11 +2538,11 @@
         <v>300</v>
       </c>
       <c r="E19" s="27" t="str">
-        <f>IF(D19="","",IF(D19=Klíč!A30,"✓","✗"))</f>
+        <f>IF(D19="","",IF(NOT(_xlfn.ISFORMULA(D19)),"✗",IF(D19=Klíč!A30,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="28" t="s">
         <v>106</v>
       </c>
@@ -2575,11 +2554,11 @@
         <v>406</v>
       </c>
       <c r="E20" s="27" t="str">
-        <f>IF(D20="","",IF(D20=Klíč!A31,"✓","✗"))</f>
+        <f>IF(D20="","",IF(NOT(_xlfn.ISFORMULA(D20)),"✗",IF(D20=Klíč!A31,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="22" spans="2:5" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B22" s="8" t="s">
         <v>77</v>
       </c>
@@ -2618,19 +2597,19 @@
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="15.36328125" customWidth="1"/>
+    <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
     <col min="4" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AB1" s="19">
         <f>COUNTIF(F15:F22,"✓")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="2:28" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="6" t="s">
         <v>108</v>
       </c>
@@ -2644,7 +2623,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>44</v>
       </c>
@@ -2655,7 +2634,7 @@
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
     </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="9" t="s">
         <v>109</v>
       </c>
@@ -2666,7 +2645,7 @@
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="4" t="s">
         <v>110</v>
       </c>
@@ -2677,7 +2656,7 @@
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
     </row>
-    <row r="8" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20" t="s">
         <v>111</v>
       </c>
@@ -2691,7 +2670,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="21" t="s">
         <v>115</v>
       </c>
@@ -2705,7 +2684,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="10" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="21" t="s">
         <v>116</v>
       </c>
@@ -2719,7 +2698,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="11" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="21" t="s">
         <v>117</v>
       </c>
@@ -2733,12 +2712,12 @@
         <v>580</v>
       </c>
     </row>
-    <row r="13" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="14" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="20" t="s">
         <v>81</v>
       </c>
@@ -2752,7 +2731,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="28" t="s">
         <v>84</v>
       </c>
@@ -2763,15 +2742,14 @@
         <v>115</v>
       </c>
       <c r="E15" s="26">
-        <f>C9*E9/100</f>
         <v>29.25</v>
       </c>
       <c r="F15" s="27" t="str">
-        <f>IF(E15="","",IF(ROUND(E15,2)=ROUND(Klíč!A40,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="16" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(E15="","",IF(NOT(_xlfn.ISFORMULA(E15)),"✗",IF(ROUND(E15,2)=ROUND(Klíč!A40,2),"✓","✗")))</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="16" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="28" t="s">
         <v>86</v>
       </c>
@@ -2782,15 +2760,14 @@
         <v>116</v>
       </c>
       <c r="E16" s="26">
-        <f>C10*E10/100</f>
         <v>16.64</v>
       </c>
       <c r="F16" s="27" t="str">
-        <f>IF(E16="","",IF(ROUND(E16,2)=ROUND(Klíč!A41,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="17" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(E16="","",IF(NOT(_xlfn.ISFORMULA(E16)),"✗",IF(ROUND(E16,2)=ROUND(Klíč!A41,2),"✓","✗")))</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="28" t="s">
         <v>88</v>
       </c>
@@ -2800,16 +2777,13 @@
       <c r="D17" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="E17" s="26">
-        <f>C9*D9*E9/100</f>
-        <v>1111.5</v>
-      </c>
+      <c r="E17" s="26"/>
       <c r="F17" s="27" t="str">
-        <f>IF(E17="","",IF(ROUND(E17,2)=ROUND(Klíč!A42,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(E17="","",IF(NOT(_xlfn.ISFORMULA(E17)),"✗",IF(ROUND(E17,2)=ROUND(Klíč!A42,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="28" t="s">
         <v>90</v>
       </c>
@@ -2819,16 +2793,13 @@
       <c r="D18" s="31" t="s">
         <v>117</v>
       </c>
-      <c r="E18" s="26">
-        <f>C11*D11*E11/100</f>
-        <v>1719.12</v>
-      </c>
+      <c r="E18" s="26"/>
       <c r="F18" s="27" t="str">
-        <f>IF(E18="","",IF(ROUND(E18,2)=ROUND(Klíč!A43,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(E18="","",IF(NOT(_xlfn.ISFORMULA(E18)),"✗",IF(ROUND(E18,2)=ROUND(Klíč!A43,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="28" t="s">
         <v>92</v>
       </c>
@@ -2838,16 +2809,13 @@
       <c r="D19" s="31" t="s">
         <v>127</v>
       </c>
-      <c r="E19" s="26">
-        <f>E11-E10</f>
-        <v>260</v>
-      </c>
+      <c r="E19" s="26"/>
       <c r="F19" s="27" t="str">
-        <f>IF(E19="","",IF(ROUND(E19,2)=ROUND(Klíč!A44,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(E19="","",IF(NOT(_xlfn.ISFORMULA(E19)),"✗",IF(ROUND(E19,2)=ROUND(Klíč!A44,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="28" t="s">
         <v>94</v>
       </c>
@@ -2857,16 +2825,13 @@
       <c r="D20" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="E20" s="26">
-        <f>(C9+C10+C11)/3</f>
-        <v>6.5</v>
-      </c>
+      <c r="E20" s="26"/>
       <c r="F20" s="27" t="str">
-        <f>IF(E20="","",IF(ROUND(E20,2)=ROUND(Klíč!A45,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(E20="","",IF(NOT(_xlfn.ISFORMULA(E20)),"✗",IF(ROUND(E20,2)=ROUND(Klíč!A45,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="28" t="s">
         <v>96</v>
       </c>
@@ -2876,16 +2841,13 @@
       <c r="D21" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="E21" s="26">
-        <f>C9*D9/100</f>
-        <v>2.4700000000000002</v>
-      </c>
+      <c r="E21" s="26"/>
       <c r="F21" s="27" t="str">
-        <f>IF(E21="","",IF(ROUND(E21,2)=ROUND(Klíč!A46,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(E21="","",IF(NOT(_xlfn.ISFORMULA(E21)),"✗",IF(ROUND(E21,2)=ROUND(Klíč!A46,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="28" t="s">
         <v>98</v>
       </c>
@@ -2895,23 +2857,20 @@
       <c r="D22" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="E22" s="26">
-        <f>C10*D10/100</f>
-        <v>2.1320000000000001</v>
-      </c>
+      <c r="E22" s="26"/>
       <c r="F22" s="27" t="str">
-        <f>IF(E22="","",IF(ROUND(E22,2)=ROUND(Klíč!A47,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+        <f>IF(E22="","",IF(NOT(_xlfn.ISFORMULA(E22)),"✗",IF(ROUND(E22,2)=ROUND(Klíč!A47,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="32" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="9" t="s">
-        <v>213</v>
+        <v>133</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
@@ -2920,9 +2879,9 @@
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="17" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2943,7 +2902,7 @@
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
     </row>
-    <row r="30" spans="2:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B30" s="8" t="s">
         <v>77</v>
       </c>
@@ -2951,7 +2910,7 @@
       <c r="D30" s="8"/>
       <c r="E30" s="7" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>8 / 8  bodů</v>
+        <v>0 / 8  bodů</v>
       </c>
       <c r="F30" s="7"/>
     </row>
@@ -2993,15 +2952,15 @@
     <col min="9" max="9" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AB1" s="19">
         <f>COUNTIF(I9:I16,"✓")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="2:28" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -3012,7 +2971,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>44</v>
       </c>
@@ -3022,9 +2981,9 @@
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
     </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -3032,26 +2991,26 @@
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
     </row>
-    <row r="7" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G8" s="20" t="s">
         <v>119</v>
@@ -3060,9 +3019,9 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="21" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C9" s="33">
         <v>1450</v>
@@ -3074,20 +3033,19 @@
         <v>320</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H9" s="34">
-        <f>SUM(C9:C22)</f>
         <v>21610</v>
       </c>
       <c r="I9" s="27" t="str">
-        <f>IF(H9="","",IF(H9=Klíč!A60,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="10" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(H9="","",IF(NOT(_xlfn.ISFORMULA(H9)),"✗",IF(H9=Klíč!A60,"✓","✗")))</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="10" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="21" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C10" s="33">
         <v>1320</v>
@@ -3099,20 +3057,20 @@
         <v>410</v>
       </c>
       <c r="G10" s="30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H10" s="34">
         <f>SUM(D9:D22)</f>
         <v>10950</v>
       </c>
       <c r="I10" s="27" t="str">
-        <f>IF(H10="","",IF(H10=Klíč!A61,"✓","✗"))</f>
+        <f>IF(H10="","",IF(NOT(_xlfn.ISFORMULA(H10)),"✗",IF(H10=Klíč!A61,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="11" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="21" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C11" s="33">
         <v>1580</v>
@@ -3124,20 +3082,20 @@
         <v>380</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H11" s="34">
         <f>SUM(E9:E22)</f>
         <v>6040</v>
       </c>
       <c r="I11" s="27" t="str">
-        <f>IF(H11="","",IF(H11=Klíč!A62,"✓","✗"))</f>
+        <f>IF(H11="","",IF(NOT(_xlfn.ISFORMULA(H11)),"✗",IF(H11=Klíč!A62,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="12" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="21" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C12" s="33">
         <v>1280</v>
@@ -3149,20 +3107,17 @@
         <v>290</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="H12" s="34">
-        <f>SUM(C9:E15)</f>
-        <v>18910</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="H12" s="34"/>
       <c r="I12" s="27" t="str">
-        <f>IF(H12="","",IF(H12=Klíč!A63,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="13" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(H12="","",IF(NOT(_xlfn.ISFORMULA(H12)),"✗",IF(H12=Klíč!A63,"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="21" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C13" s="33">
         <v>1820</v>
@@ -3174,20 +3129,17 @@
         <v>540</v>
       </c>
       <c r="G13" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="H13" s="34">
-        <f>SUM(C16:E22)</f>
-        <v>19690</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="H13" s="34"/>
       <c r="I13" s="27" t="str">
-        <f>IF(H13="","",IF(H13=Klíč!A64,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="14" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(H13="","",IF(NOT(_xlfn.ISFORMULA(H13)),"✗",IF(H13=Klíč!A64,"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C14" s="33">
         <v>2150</v>
@@ -3199,20 +3151,17 @@
         <v>720</v>
       </c>
       <c r="G14" s="30" t="s">
-        <v>153</v>
-      </c>
-      <c r="H14" s="34">
-        <f>SUM(C14:E15)</f>
-        <v>5760</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="H14" s="34"/>
       <c r="I14" s="27" t="str">
-        <f>IF(H14="","",IF(H14=Klíč!A65,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="15" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(H14="","",IF(NOT(_xlfn.ISFORMULA(H14)),"✗",IF(H14=Klíč!A65,"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C15" s="33">
         <v>980</v>
@@ -3224,20 +3173,17 @@
         <v>280</v>
       </c>
       <c r="G15" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="H15" s="34">
-        <f>SUM(C21:E22)</f>
-        <v>6100</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="H15" s="34"/>
       <c r="I15" s="27" t="str">
-        <f>IF(H15="","",IF(H15=Klíč!A66,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="16" spans="2:28" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(H15="","",IF(NOT(_xlfn.ISFORMULA(H15)),"✗",IF(H15=Klíč!A66,"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="21" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C16" s="33">
         <v>1390</v>
@@ -3249,20 +3195,17 @@
         <v>350</v>
       </c>
       <c r="G16" s="30" t="s">
-        <v>157</v>
-      </c>
-      <c r="H16" s="34">
-        <f>SUM(C9,C16)</f>
-        <v>2840</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="H16" s="34"/>
       <c r="I16" s="27" t="str">
-        <f>IF(H16="","",IF(H16=Klíč!A67,"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
+        <f>IF(H16="","",IF(NOT(_xlfn.ISFORMULA(H16)),"✗",IF(H16=Klíč!A67,"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="21" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C17" s="33">
         <v>1450</v>
@@ -3274,9 +3217,9 @@
         <v>390</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="21" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C18" s="33">
         <v>1620</v>
@@ -3288,9 +3231,9 @@
         <v>420</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="21" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C19" s="33">
         <v>1340</v>
@@ -3302,9 +3245,9 @@
         <v>310</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="21" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C20" s="33">
         <v>1900</v>
@@ -3316,9 +3259,9 @@
         <v>580</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C21" s="33">
         <v>2280</v>
@@ -3330,9 +3273,9 @@
         <v>760</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C22" s="33">
         <v>1050</v>
@@ -3344,7 +3287,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="25" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B25" s="8" t="s">
         <v>77</v>
       </c>
@@ -3353,7 +3296,7 @@
       <c r="E25" s="8"/>
       <c r="F25" s="7" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>8 / 8  bodů</v>
+        <v>2 / 8  bodů</v>
       </c>
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
@@ -3386,22 +3329,22 @@
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="44.36328125" customWidth="1"/>
+    <col min="2" max="2" width="6" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="15.7265625" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AB1" s="19">
         <f>COUNTIF(F19:F28,"✓")</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="2:28" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -3412,7 +3355,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>44</v>
       </c>
@@ -3422,9 +3365,9 @@
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
     </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -3432,9 +3375,9 @@
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
@@ -3442,26 +3385,26 @@
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="8" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="9" spans="2:28" x14ac:dyDescent="0.35">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C9" s="22">
         <v>22</v>
@@ -3476,9 +3419,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="21" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C10" s="22">
         <v>25</v>
@@ -3493,9 +3436,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="21" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C11" s="22">
         <v>28</v>
@@ -3510,9 +3453,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="21" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C12" s="22">
         <v>31</v>
@@ -3527,9 +3470,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C13" s="22">
         <v>29</v>
@@ -3544,9 +3487,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C14" s="22">
         <v>24</v>
@@ -3561,9 +3504,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" s="22">
         <v>19</v>
@@ -3578,17 +3521,17 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="2:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="24" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" ht="15.5" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="20" t="s">
         <v>81</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D18" s="20" t="s">
         <v>121</v>
@@ -3597,32 +3540,28 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="28" t="s">
         <v>84</v>
       </c>
       <c r="C19" s="30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D19" s="35">
-        <f>AVERAGE(C9:C15)</f>
-        <v>25.428571428571427</v>
-      </c>
-      <c r="E19" s="36">
-        <f>D19</f>
-        <v>25.428571428571427</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E19" s="36"/>
       <c r="F19" s="27" t="str">
-        <f>IF(E19="","",IF(ROUND(E19,2)=ROUND(Klíč!A80,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(AND(D19="",E19=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D19)),NOT(_xlfn.ISFORMULA(E19))),"✗",IF(AND(ROUND(D19,2)=ROUND(Klíč!A80,2),ROUND(E19,2)=ROUND(Klíč!A80,2)),"✓","✗")))</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="28" t="s">
         <v>86</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D20" s="35">
         <f>MAX(D9:D15)</f>
@@ -3633,171 +3572,123 @@
         <v>32</v>
       </c>
       <c r="F20" s="27" t="str">
-        <f>IF(E20="","",IF(ROUND(E20,2)=ROUND(Klíč!A81,2),"✓","✗"))</f>
+        <f>IF(AND(D20="",E20=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D20)),NOT(_xlfn.ISFORMULA(E20))),"✗",IF(AND(ROUND(D20,2)=ROUND(Klíč!A81,2),ROUND(E20,2)=ROUND(Klíč!A81,2)),"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
-    <row r="21" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="28" t="s">
         <v>88</v>
       </c>
       <c r="C21" s="30" t="s">
-        <v>176</v>
-      </c>
-      <c r="D21" s="35">
-        <f>MIN(E9:E15)</f>
-        <v>18</v>
-      </c>
-      <c r="E21" s="36">
-        <f>D21</f>
-        <v>18</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="D21" s="35"/>
+      <c r="E21" s="36"/>
       <c r="F21" s="27" t="str">
-        <f>IF(E21="","",IF(ROUND(E21,2)=ROUND(Klíč!A82,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(AND(D21="",E21=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D21)),NOT(_xlfn.ISFORMULA(E21))),"✗",IF(AND(ROUND(D21,2)=ROUND(Klíč!A82,2),ROUND(E21,2)=ROUND(Klíč!A82,2)),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="28" t="s">
         <v>90</v>
       </c>
       <c r="C22" s="30" t="s">
-        <v>177</v>
-      </c>
-      <c r="D22" s="35">
-        <f>AVERAGE(F9:F15)</f>
-        <v>25.571428571428573</v>
-      </c>
-      <c r="E22" s="36">
-        <f>D22</f>
-        <v>25.571428571428573</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="D22" s="35"/>
+      <c r="E22" s="36"/>
       <c r="F22" s="27" t="str">
-        <f>IF(E22="","",IF(ROUND(E22,2)=ROUND(Klíč!A83,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(AND(D22="",E22=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D22)),NOT(_xlfn.ISFORMULA(E22))),"✗",IF(AND(ROUND(D22,2)=ROUND(Klíč!A83,2),ROUND(E22,2)=ROUND(Klíč!A83,2)),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="28" t="s">
         <v>92</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>178</v>
-      </c>
-      <c r="D23" s="35">
-        <f>MAX(C9:F15)</f>
-        <v>32</v>
-      </c>
-      <c r="E23" s="36">
-        <f>D23</f>
-        <v>32</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="D23" s="35"/>
+      <c r="E23" s="36"/>
       <c r="F23" s="27" t="str">
-        <f>IF(E23="","",IF(ROUND(E23,2)=ROUND(Klíč!A84,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(AND(D23="",E23=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D23)),NOT(_xlfn.ISFORMULA(E23))),"✗",IF(AND(ROUND(D23,2)=ROUND(Klíč!A84,2),ROUND(E23,2)=ROUND(Klíč!A84,2)),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="28" t="s">
         <v>94</v>
       </c>
       <c r="C24" s="30" t="s">
-        <v>179</v>
-      </c>
-      <c r="D24" s="35">
-        <f>MIN(C9:F15)</f>
-        <v>18</v>
-      </c>
-      <c r="E24" s="36">
-        <f>D24</f>
-        <v>18</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="D24" s="35"/>
+      <c r="E24" s="36"/>
       <c r="F24" s="27" t="str">
-        <f>IF(E24="","",IF(ROUND(E24,2)=ROUND(Klíč!A85,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(AND(D24="",E24=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D24)),NOT(_xlfn.ISFORMULA(E24))),"✗",IF(AND(ROUND(D24,2)=ROUND(Klíč!A85,2),ROUND(E24,2)=ROUND(Klíč!A85,2)),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="28" t="s">
         <v>96</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>180</v>
-      </c>
-      <c r="D25" s="35">
-        <f>COUNT(C9:F15)</f>
-        <v>28</v>
-      </c>
-      <c r="E25" s="36">
-        <f>D25</f>
-        <v>28</v>
-      </c>
+        <v>181</v>
+      </c>
+      <c r="D25" s="35"/>
+      <c r="E25" s="36"/>
       <c r="F25" s="27" t="str">
-        <f>IF(E25="","",IF(ROUND(E25,2)=ROUND(Klíč!A86,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(AND(D25="",E25=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D25)),NOT(_xlfn.ISFORMULA(E25))),"✗",IF(AND(ROUND(D25,2)=ROUND(Klíč!A86,2),ROUND(E25,2)=ROUND(Klíč!A86,2)),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="28" t="s">
         <v>98</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>181</v>
-      </c>
-      <c r="D26" s="35">
-        <f>AVERAGE(C12:F12)</f>
-        <v>30.75</v>
-      </c>
-      <c r="E26" s="36">
-        <f>D26</f>
-        <v>30.75</v>
-      </c>
+        <v>182</v>
+      </c>
+      <c r="D26" s="35"/>
+      <c r="E26" s="36"/>
       <c r="F26" s="27" t="str">
-        <f>IF(E26="","",IF(ROUND(E26,2)=ROUND(Klíč!A87,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(AND(D26="",E26=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D26)),NOT(_xlfn.ISFORMULA(E26))),"✗",IF(AND(ROUND(D26,2)=ROUND(Klíč!A87,2),ROUND(E26,2)=ROUND(Klíč!A87,2)),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="28" t="s">
         <v>100</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="D27" s="35">
-        <f>MAX(C9:C15)-MIN(C9:C15)</f>
-        <v>12</v>
-      </c>
-      <c r="E27" s="36">
-        <f>D27</f>
-        <v>12</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="D27" s="35"/>
+      <c r="E27" s="36"/>
       <c r="F27" s="27" t="str">
-        <f>IF(E27="","",IF(ROUND(E27,2)=ROUND(Klíč!A88,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(AND(D27="",E27=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D27)),NOT(_xlfn.ISFORMULA(E27))),"✗",IF(AND(ROUND(D27,2)=ROUND(Klíč!A88,2),ROUND(E27,2)=ROUND(Klíč!A88,2)),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="28" t="s">
         <v>102</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>183</v>
-      </c>
-      <c r="D28" s="35">
-        <f>SUM(D9:D15)</f>
-        <v>187</v>
-      </c>
-      <c r="E28" s="36">
-        <f>D28</f>
-        <v>187</v>
-      </c>
+        <v>184</v>
+      </c>
+      <c r="D28" s="35"/>
+      <c r="E28" s="36"/>
       <c r="F28" s="27" t="str">
-        <f>IF(E28="","",IF(ROUND(E28,2)=ROUND(Klíč!A89,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" ht="18.5" x14ac:dyDescent="0.45">
+        <f>IF(AND(D28="",E28=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D28)),NOT(_xlfn.ISFORMULA(E28))),"✗",IF(AND(ROUND(D28,2)=ROUND(Klíč!A89,2),ROUND(E28,2)=ROUND(Klíč!A89,2)),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B30" s="8" t="s">
         <v>77</v>
       </c>
@@ -3805,7 +3696,7 @@
       <c r="D30" s="8"/>
       <c r="E30" s="7" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>10 / 10  bodů</v>
+        <v>1 / 10  bodů</v>
       </c>
       <c r="F30" s="7"/>
     </row>
@@ -3838,23 +3729,19 @@
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" customWidth="1"/>
-    <col min="4" max="4" width="25.6328125" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16.453125" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="3" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AB1" s="19">
         <f>COUNTIF(G20:G27,"✓")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="2:28" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -3866,7 +3753,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>44</v>
       </c>
@@ -3877,9 +3764,9 @@
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
     </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -3888,9 +3775,9 @@
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
@@ -3899,29 +3786,29 @@
       <c r="G6" s="9"/>
       <c r="H6" s="9"/>
     </row>
-    <row r="8" spans="2:28" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="9" spans="2:28" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="21" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C9" s="22">
         <v>11.8</v>
@@ -3939,9 +3826,9 @@
         <v>285</v>
       </c>
     </row>
-    <row r="10" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C10" s="22">
         <v>12.2</v>
@@ -3959,9 +3846,9 @@
         <v>295</v>
       </c>
     </row>
-    <row r="11" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="21" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C11" s="22">
         <v>11.5</v>
@@ -3979,9 +3866,9 @@
         <v>278</v>
       </c>
     </row>
-    <row r="12" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="21" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C12" s="22">
         <v>12.5</v>
@@ -3999,9 +3886,9 @@
         <v>310</v>
       </c>
     </row>
-    <row r="13" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="21" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C13" s="22">
         <v>11.9</v>
@@ -4019,9 +3906,9 @@
         <v>290</v>
       </c>
     </row>
-    <row r="14" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="21" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C14" s="22">
         <v>12</v>
@@ -4039,9 +3926,9 @@
         <v>298</v>
       </c>
     </row>
-    <row r="15" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="21" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C15" s="22">
         <v>11.7</v>
@@ -4059,9 +3946,9 @@
         <v>282</v>
       </c>
     </row>
-    <row r="16" spans="2:28" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="21" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C16" s="22">
         <v>12.3</v>
@@ -4079,12 +3966,12 @@
         <v>305</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="24" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="20" t="s">
         <v>81</v>
       </c>
@@ -4092,156 +3979,132 @@
         <v>119</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="28" t="s">
         <v>84</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="F20" s="36">
-        <f>AVERAGE(C9:C16)</f>
-        <v>11.987500000000001</v>
-      </c>
+      <c r="F20" s="36"/>
       <c r="G20" s="27" t="str">
-        <f>IF(F20="","",IF(ROUND(F20,2)=ROUND(Klíč!A100,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(F20="","",IF(NOT(_xlfn.ISFORMULA(F20)),"✗",IF(ROUND(F20,2)=ROUND(Klíč!A100,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="28" t="s">
         <v>86</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
-      <c r="F21" s="36">
-        <f>MIN(C9:C16)</f>
-        <v>11.5</v>
-      </c>
+      <c r="F21" s="36"/>
       <c r="G21" s="27" t="str">
-        <f>IF(F21="","",IF(ROUND(F21,2)=ROUND(Klíč!A101,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(F21="","",IF(NOT(_xlfn.ISFORMULA(F21)),"✗",IF(ROUND(F21,2)=ROUND(Klíč!A101,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="28" t="s">
         <v>88</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
-      <c r="F22" s="36">
-        <f>MAX(D9:D16)</f>
-        <v>7.1</v>
-      </c>
+      <c r="F22" s="36"/>
       <c r="G22" s="27" t="str">
-        <f>IF(F22="","",IF(ROUND(F22,2)=ROUND(Klíč!A102,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="23" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(F22="","",IF(NOT(_xlfn.ISFORMULA(F22)),"✗",IF(ROUND(F22,2)=ROUND(Klíč!A102,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="28" t="s">
         <v>90</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
-      <c r="F23" s="36">
-        <f>AVERAGE(E9:E16)</f>
-        <v>13.074999999999999</v>
-      </c>
+      <c r="F23" s="36"/>
       <c r="G23" s="27" t="str">
-        <f>IF(F23="","",IF(ROUND(F23,2)=ROUND(Klíč!A103,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(F23="","",IF(NOT(_xlfn.ISFORMULA(F23)),"✗",IF(ROUND(F23,2)=ROUND(Klíč!A103,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="28" t="s">
         <v>92</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
-      <c r="F24" s="36">
-        <f>MAX(F9:F16)-MIN(F9:F16)</f>
-        <v>0.16999999999999993</v>
-      </c>
+      <c r="F24" s="36"/>
       <c r="G24" s="27" t="str">
-        <f>IF(F24="","",IF(ROUND(F24,2)=ROUND(Klíč!A104,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(F24="","",IF(NOT(_xlfn.ISFORMULA(F24)),"✗",IF(ROUND(F24,2)=ROUND(Klíč!A104,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="28" t="s">
         <v>94</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
-      <c r="F25" s="36">
-        <f>SUM(G9:G16)</f>
-        <v>2343</v>
-      </c>
+      <c r="F25" s="36"/>
       <c r="G25" s="27" t="str">
-        <f>IF(F25="","",IF(ROUND(F25,2)=ROUND(Klíč!A105,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(F25="","",IF(NOT(_xlfn.ISFORMULA(F25)),"✗",IF(ROUND(F25,2)=ROUND(Klíč!A105,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="28" t="s">
         <v>96</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
-      <c r="F26" s="36">
-        <f>AVERAGE(G9,G11,G15)</f>
-        <v>281.66666666666669</v>
-      </c>
+      <c r="F26" s="36"/>
       <c r="G26" s="27" t="str">
-        <f>IF(F26="","",IF(ROUND(F26,2)=ROUND(Klíč!A106,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="27" spans="2:8" ht="18.5" x14ac:dyDescent="0.35">
+        <f>IF(F26="","",IF(NOT(_xlfn.ISFORMULA(F26)),"✗",IF(ROUND(F26,2)=ROUND(Klíč!A106,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="28" t="s">
         <v>98</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
-      <c r="F27" s="36">
-        <f>COUNT(C9:C16)</f>
-        <v>8</v>
-      </c>
+      <c r="F27" s="36"/>
       <c r="G27" s="27" t="str">
-        <f>IF(F27="","",IF(ROUND(F27,2)=ROUND(Klíč!A107,2),"✓","✗"))</f>
-        <v>✓</v>
-      </c>
-    </row>
-    <row r="29" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+        <f>IF(F27="","",IF(NOT(_xlfn.ISFORMULA(F27)),"✗",IF(ROUND(F27,2)=ROUND(Klíč!A107,2),"✓","✗")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -4250,9 +4113,9 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
@@ -4288,7 +4151,7 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
     </row>
-    <row r="35" spans="2:8" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B35" s="8" t="s">
         <v>77</v>
       </c>
@@ -4296,7 +4159,7 @@
       <c r="D35" s="8"/>
       <c r="E35" s="7" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>8 / 8  bodů</v>
+        <v>0 / 8  bodů</v>
       </c>
       <c r="F35" s="7"/>
       <c r="G35" s="7"/>

</xml_diff>

<commit_message>
Oprava klíče Úkolu 4 — tři špatné hodnoty součtů
Úkol 4, Klíč: A60 22610→21610, A63 22660→18910, A64 16940→19690

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/answer_keys/03_Uvod_HZD.xlsx
+++ b/data/answer_keys/03_Uvod_HZD.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip.senkerik\Desktop\Aplikace pro opravu excel souborů\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849254C3-0DFF-49DA-A848-8E74E2691AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4934C36C-4136-48D2-BCFE-D095990D85B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pokyny" sheetId="1" r:id="rId1"/>
-    <sheet name="Klíč" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Klíč" sheetId="2" r:id="rId2"/>
     <sheet name="Úkol 1" sheetId="3" r:id="rId3"/>
     <sheet name="Úkol 2" sheetId="4" r:id="rId4"/>
     <sheet name="Úkol 3" sheetId="5" r:id="rId5"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="215">
   <si>
     <t>Hromadné zpracování dat – Cvičení (1. hodina)</t>
   </si>
@@ -691,6 +691,12 @@
   </si>
   <si>
     <t>Který z těchto závodníků by byl podle tebe nejlepší ve víceboji a proč?</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>Na dvě des. místa</t>
   </si>
 </sst>
 </file>
@@ -905,22 +911,8 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -940,7 +932,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -954,9 +945,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -975,6 +963,24 @@
     <xf numFmtId="2" fontId="15" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -1335,239 +1341,249 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
     </row>
     <row r="5" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
     </row>
     <row r="8" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
     </row>
     <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
     </row>
     <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
     </row>
     <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
     </row>
     <row r="17" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
     </row>
     <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
     </row>
     <row r="21" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
     </row>
     <row r="22" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
     </row>
     <row r="23" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
     </row>
     <row r="24" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
     </row>
     <row r="27" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="7" t="str">
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="30" t="str">
         <f>SUM('Úkol 1'!AB1,'Úkol 2'!AB1,'Úkol 3'!AB1,'Úkol 4'!AB1,'Úkol 5'!AB1,'Úkol 6'!AB1) &amp; " / " &amp; SUM('Úkol 1'!AB2,'Úkol 2'!AB2,'Úkol 3'!AB2,'Úkol 4'!AB2,'Úkol 5'!AB2,'Úkol 6'!AB2)</f>
-        <v>17 / 56</v>
-      </c>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
+        <v>56 / 56</v>
+      </c>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="C13:H13"/>
+    <mergeCell ref="C14:H14"/>
+    <mergeCell ref="C15:H15"/>
     <mergeCell ref="D24:H24"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="E27:H27"/>
@@ -1576,16 +1592,6 @@
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D22:H22"/>
     <mergeCell ref="D23:H23"/>
-    <mergeCell ref="C11:H11"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="C13:H13"/>
-    <mergeCell ref="C14:H14"/>
-    <mergeCell ref="C15:H15"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="C10:H10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1598,7 +1604,7 @@
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="8" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1729,7 +1735,7 @@
     </row>
     <row r="43" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43">
-        <v>1718.16</v>
+        <v>1719.12</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1754,7 +1760,7 @@
     </row>
     <row r="60" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60">
-        <v>22610</v>
+        <v>21610</v>
       </c>
     </row>
     <row r="61" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1769,12 +1775,12 @@
     </row>
     <row r="63" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63">
-        <v>22660</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="64" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64">
-        <v>16940</v>
+        <v>19690</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1894,7 +1900,7 @@
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="6" customWidth="1"/>
+    <col min="2" max="2" width="15.36328125" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
@@ -1902,384 +1908,404 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="AB1" s="19">
+      <c r="AB1" s="9">
         <f>COUNTIF(H17:H26,"✓")</f>
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="AB2" s="19">
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="AB2" s="9">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
     </row>
     <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
     </row>
     <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="10" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="9" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="12">
         <v>18</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="12">
         <v>18</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="12">
         <v>19</v>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="13">
         <f t="shared" ref="F9:F14" si="0">AVERAGE(C9:E9)</f>
         <v>18.333333333333332</v>
       </c>
     </row>
     <row r="10" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="12">
         <v>25</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="12">
         <v>24</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="12">
         <v>23</v>
       </c>
-      <c r="F10" s="23">
+      <c r="F10" s="13">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="12">
         <v>15</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="12">
         <v>18</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="12">
         <v>20</v>
       </c>
-      <c r="F11" s="23">
+      <c r="F11" s="13">
         <f t="shared" si="0"/>
         <v>17.666666666666668</v>
       </c>
     </row>
     <row r="12" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="12">
         <v>22</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="12">
         <v>21</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="12">
         <v>24</v>
       </c>
-      <c r="F12" s="23">
+      <c r="F12" s="13">
         <f t="shared" si="0"/>
         <v>22.333333333333332</v>
       </c>
     </row>
     <row r="13" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="12">
         <v>17</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="12">
         <v>19</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="12">
         <v>18</v>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="13">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
     <row r="14" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="12">
         <v>19</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="12">
         <v>16</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="12">
         <v>18</v>
       </c>
-      <c r="F14" s="23">
+      <c r="F14" s="13">
         <f t="shared" si="0"/>
         <v>17.666666666666668</v>
       </c>
     </row>
     <row r="16" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="1" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="26">
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="15">
         <v>25</v>
       </c>
-      <c r="H17" s="27" t="str">
+      <c r="H17" s="16" t="str">
         <f>IF(G17="","",IF(G17=Klíč!A2,"✓","✗"))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="26">
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="15">
         <v>20</v>
       </c>
-      <c r="H18" s="27" t="str">
+      <c r="H18" s="16" t="str">
         <f>IF(G18="","",IF(G18=Klíč!A3,"✓","✗"))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="27" t="str">
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="15" t="str">
+        <f>B12</f>
+        <v>Dana</v>
+      </c>
+      <c r="H19" s="16" t="str">
         <f>IF(TRIM(LOWER(G19))="","",IF(TRIM(LOWER(G19))=TRIM(LOWER(Klíč!A4)),"✓","✗"))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="27" t="str">
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="15">
+        <f>D12</f>
+        <v>21</v>
+      </c>
+      <c r="H20" s="16" t="str">
         <f>IF(G20="","",IF(G20=Klíč!A5,"✓","✗"))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="27" t="str">
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="15" t="str">
+        <f>B14</f>
+        <v>Filip</v>
+      </c>
+      <c r="H21" s="16" t="str">
         <f>IF(TRIM(LOWER(G21))="","",IF(TRIM(LOWER(G21))=TRIM(LOWER(Klíč!A6)),"✓","✗"))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="27" t="str">
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="15">
+        <f>D9</f>
+        <v>18</v>
+      </c>
+      <c r="H22" s="16" t="str">
         <f>IF(G22="","",IF(G22=Klíč!A7,"✓","✗"))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="25" t="s">
+      <c r="B23" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="27" t="str">
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="H23" s="16" t="str">
         <f>IF(TRIM(LOWER(G23))="","",IF(TRIM(LOWER(G23))=TRIM(LOWER(Klíč!A8)),"✓","✗"))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="25" t="s">
+      <c r="B24" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="27" t="str">
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H24" s="16" t="str">
         <f>IF(TRIM(LOWER(G24))="","",IF(TRIM(LOWER(G24))=TRIM(LOWER(Klíč!A9)),"✓","✗"))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="27" t="str">
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="15">
+        <v>13</v>
+      </c>
+      <c r="H25" s="16" t="str">
         <f>IF(G25="","",IF(G25=Klíč!A10,"✓","✗"))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="25" t="s">
+      <c r="B26" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="27" t="str">
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="H26" s="16" t="str">
         <f>IF(TRIM(LOWER(G26))="","",IF(TRIM(LOWER(G26))=TRIM(LOWER(Klíč!A11)),"✓","✗"))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="28" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="7" t="str">
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="30" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>2 / 10  bodů</v>
-      </c>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
+        <v>10 / 10  bodů</v>
+      </c>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C22:F22"/>
     <mergeCell ref="C23:F23"/>
     <mergeCell ref="C24:F24"/>
     <mergeCell ref="C25:F25"/>
     <mergeCell ref="C26:F26"/>
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="F28:H28"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="C17:F17"/>
   </mergeCells>
   <conditionalFormatting sqref="H17:H26">
     <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
@@ -2307,267 +2333,267 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="AB1" s="19">
+      <c r="AB1" s="9">
         <f>COUNTIF(E9:E20,"✓")</f>
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="AB2" s="19">
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="AB2" s="9">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
     </row>
     <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
     </row>
     <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
     </row>
     <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="10" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="9" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="15">
         <f>145+287</f>
         <v>432</v>
       </c>
-      <c r="E9" s="27" t="str">
+      <c r="E9" s="16" t="str">
         <f>IF(D9="","",IF(NOT(_xlfn.ISFORMULA(D9)),"✗",IF(D9=Klíč!A20,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="10" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="15">
         <f>1000-437</f>
         <v>563</v>
       </c>
-      <c r="E10" s="27" t="str">
+      <c r="E10" s="16" t="str">
         <f>IF(D10="","",IF(NOT(_xlfn.ISFORMULA(D10)),"✗",IF(D10=Klíč!A21,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="11" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="15">
         <f>17*23</f>
         <v>391</v>
       </c>
-      <c r="E11" s="27" t="str">
+      <c r="E11" s="16" t="str">
         <f>IF(D11="","",IF(NOT(_xlfn.ISFORMULA(D11)),"✗",IF(D11=Klíč!A22,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="12" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="15">
         <f>1024/16</f>
         <v>64</v>
       </c>
-      <c r="E12" s="27" t="str">
+      <c r="E12" s="16" t="str">
         <f>IF(D12="","",IF(NOT(_xlfn.ISFORMULA(D12)),"✗",IF(D12=Klíč!A23,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="13" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="15">
         <f>(45+55)*8</f>
         <v>800</v>
       </c>
-      <c r="E13" s="27" t="str">
+      <c r="E13" s="16" t="str">
         <f>IF(D13="","",IF(NOT(_xlfn.ISFORMULA(D13)),"✗",IF(D13=Klíč!A24,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="14" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="15">
         <f>2^10</f>
         <v>1024</v>
       </c>
-      <c r="E14" s="27" t="str">
+      <c r="E14" s="16" t="str">
         <f>IF(D14="","",IF(NOT(_xlfn.ISFORMULA(D14)),"✗",IF(D14=Klíč!A25,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="15" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C15" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="15">
         <f>(250-50)/(2+8)</f>
         <v>20</v>
       </c>
-      <c r="E15" s="27" t="str">
+      <c r="E15" s="16" t="str">
         <f>IF(D15="","",IF(NOT(_xlfn.ISFORMULA(D15)),"✗",IF(D15=Klíč!A26,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="16" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="15">
         <f>7*60+35</f>
         <v>455</v>
       </c>
-      <c r="E16" s="27" t="str">
+      <c r="E16" s="16" t="str">
         <f>IF(D16="","",IF(NOT(_xlfn.ISFORMULA(D16)),"✗",IF(D16=Klíč!A27,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="15">
         <f>12^2+5^2</f>
         <v>169</v>
       </c>
-      <c r="E17" s="27" t="str">
+      <c r="E17" s="16" t="str">
         <f>IF(D17="","",IF(NOT(_xlfn.ISFORMULA(D17)),"✗",IF(D17=Klíč!A28,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="D18" s="26">
+      <c r="D18" s="15">
         <f>365*24*60</f>
         <v>525600</v>
       </c>
-      <c r="E18" s="27" t="str">
+      <c r="E18" s="16" t="str">
         <f>IF(D18="","",IF(NOT(_xlfn.ISFORMULA(D18)),"✗",IF(D18=Klíč!A29,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C19" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="15">
         <f>800*3/4/2</f>
         <v>300</v>
       </c>
-      <c r="E19" s="27" t="str">
+      <c r="E19" s="16" t="str">
         <f>IF(D19="","",IF(NOT(_xlfn.ISFORMULA(D19)),"✗",IF(D19=Klíč!A30,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D20" s="26">
+      <c r="D20" s="15">
         <f>12*38-50</f>
         <v>406</v>
       </c>
-      <c r="E20" s="27" t="str">
+      <c r="E20" s="16" t="str">
         <f>IF(D20="","",IF(NOT(_xlfn.ISFORMULA(D20)),"✗",IF(D20=Klíč!A31,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="22" spans="2:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="7" t="str">
+      <c r="C22" s="29"/>
+      <c r="D22" s="30" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
         <v>12 / 12  bodů</v>
       </c>
-      <c r="E22" s="7"/>
+      <c r="E22" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2597,322 +2623,342 @@
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="6" customWidth="1"/>
+    <col min="2" max="2" width="14.90625" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
     <col min="4" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="AB1" s="19">
+      <c r="AB1" s="9">
         <f>COUNTIF(F15:F22,"✓")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="AB2" s="19">
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="AB2" s="9">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
     </row>
     <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
     </row>
     <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="10" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="9" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="12">
         <v>6.5</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="12">
         <v>38</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="12">
         <v>450</v>
       </c>
     </row>
     <row r="10" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="12">
         <v>5.2</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="12">
         <v>41</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="12">
         <v>320</v>
       </c>
     </row>
     <row r="11" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="12">
         <v>7.8</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="12">
         <v>38</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="12">
         <v>580</v>
       </c>
     </row>
     <row r="13" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="1" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="14" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="10" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="15" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D15" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="15">
+        <f>C9*E9/100</f>
         <v>29.25</v>
       </c>
-      <c r="F15" s="27" t="str">
+      <c r="F15" s="16" t="str">
         <f>IF(E15="","",IF(NOT(_xlfn.ISFORMULA(E15)),"✗",IF(ROUND(E15,2)=ROUND(Klíč!A40,2),"✓","✗")))</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
     </row>
     <row r="16" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="E16" s="26">
+      <c r="E16" s="15">
+        <f>C10*E10/100</f>
         <v>16.64</v>
       </c>
-      <c r="F16" s="27" t="str">
+      <c r="F16" s="16" t="str">
         <f>IF(E16="","",IF(NOT(_xlfn.ISFORMULA(E16)),"✗",IF(ROUND(E16,2)=ROUND(Klíč!A41,2),"✓","✗")))</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="C17" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D17" s="31" t="s">
+      <c r="D17" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="E17" s="26"/>
-      <c r="F17" s="27" t="str">
+      <c r="E17" s="15">
+        <f>C9*D9*E9/100</f>
+        <v>1111.5</v>
+      </c>
+      <c r="F17" s="16" t="str">
         <f>IF(E17="","",IF(NOT(_xlfn.ISFORMULA(E17)),"✗",IF(ROUND(E17,2)=ROUND(Klíč!A42,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="30" t="s">
+      <c r="C18" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D18" s="31" t="s">
+      <c r="D18" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="27" t="str">
+      <c r="E18" s="15">
+        <f>C11*D11*E11/100</f>
+        <v>1719.12</v>
+      </c>
+      <c r="F18" s="16" t="str">
         <f>IF(E18="","",IF(NOT(_xlfn.ISFORMULA(E18)),"✗",IF(ROUND(E18,2)=ROUND(Klíč!A43,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C19" s="30" t="s">
+      <c r="C19" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="D19" s="31" t="s">
+      <c r="D19" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="E19" s="26"/>
-      <c r="F19" s="27" t="str">
+      <c r="E19" s="15">
+        <f>E11-E10</f>
+        <v>260</v>
+      </c>
+      <c r="F19" s="16" t="str">
         <f>IF(E19="","",IF(NOT(_xlfn.ISFORMULA(E19)),"✗",IF(ROUND(E19,2)=ROUND(Klíč!A44,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="D20" s="31" t="s">
+      <c r="D20" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="27" t="str">
+      <c r="E20" s="15">
+        <f>(C9+C10+C11)/3</f>
+        <v>6.5</v>
+      </c>
+      <c r="F20" s="16" t="str">
         <f>IF(E20="","",IF(NOT(_xlfn.ISFORMULA(E20)),"✗",IF(ROUND(E20,2)=ROUND(Klíč!A45,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D21" s="31" t="s">
+      <c r="D21" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="E21" s="26"/>
-      <c r="F21" s="27" t="str">
+      <c r="E21" s="15">
+        <f>C9*D9/100</f>
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="F21" s="16" t="str">
         <f>IF(E21="","",IF(NOT(_xlfn.ISFORMULA(E21)),"✗",IF(ROUND(E21,2)=ROUND(Klíč!A46,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D22" s="31" t="s">
+      <c r="D22" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="E22" s="26"/>
-      <c r="F22" s="27" t="str">
+      <c r="E22" s="15">
+        <f>C10*D10/100</f>
+        <v>2.1320000000000001</v>
+      </c>
+      <c r="F22" s="16" t="str">
         <f>IF(E22="","",IF(NOT(_xlfn.ISFORMULA(E22)),"✗",IF(ROUND(E22,2)=ROUND(Klíč!A47,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="20" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
     </row>
     <row r="26" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="7" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="34"/>
     </row>
     <row r="28" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
     </row>
     <row r="30" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="7" t="str">
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="30" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>0 / 8  bodů</v>
-      </c>
-      <c r="F30" s="7"/>
+        <v>8 / 8  bodů</v>
+      </c>
+      <c r="F30" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2953,354 +2999,370 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="AB1" s="19">
+      <c r="AB1" s="9">
         <f>COUNTIF(I9:I16,"✓")</f>
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="AB2" s="19">
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="AB2" s="9">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
     </row>
     <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
     </row>
     <row r="7" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="6" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="10" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="9" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="C9" s="33">
+      <c r="C9" s="21">
         <v>1450</v>
       </c>
-      <c r="D9" s="33">
+      <c r="D9" s="21">
         <v>680</v>
       </c>
-      <c r="E9" s="33">
+      <c r="E9" s="21">
         <v>320</v>
       </c>
-      <c r="G9" s="30" t="s">
+      <c r="G9" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="H9" s="34">
+      <c r="H9" s="22">
+        <f>SUM(C9:C22)</f>
         <v>21610</v>
       </c>
-      <c r="I9" s="27" t="str">
+      <c r="I9" s="16" t="str">
         <f>IF(H9="","",IF(NOT(_xlfn.ISFORMULA(H9)),"✗",IF(H9=Klíč!A60,"✓","✗")))</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
     </row>
     <row r="10" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="C10" s="33">
+      <c r="C10" s="21">
         <v>1320</v>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="21">
         <v>720</v>
       </c>
-      <c r="E10" s="33">
+      <c r="E10" s="21">
         <v>410</v>
       </c>
-      <c r="G10" s="30" t="s">
+      <c r="G10" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H10" s="34">
+      <c r="H10" s="22">
         <f>SUM(D9:D22)</f>
         <v>10950</v>
       </c>
-      <c r="I10" s="27" t="str">
+      <c r="I10" s="16" t="str">
         <f>IF(H10="","",IF(NOT(_xlfn.ISFORMULA(H10)),"✗",IF(H10=Klíč!A61,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="11" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="C11" s="33">
+      <c r="C11" s="21">
         <v>1580</v>
       </c>
-      <c r="D11" s="33">
+      <c r="D11" s="21">
         <v>850</v>
       </c>
-      <c r="E11" s="33">
+      <c r="E11" s="21">
         <v>380</v>
       </c>
-      <c r="G11" s="30" t="s">
+      <c r="G11" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="H11" s="34">
+      <c r="H11" s="22">
         <f>SUM(E9:E22)</f>
         <v>6040</v>
       </c>
-      <c r="I11" s="27" t="str">
+      <c r="I11" s="16" t="str">
         <f>IF(H11="","",IF(NOT(_xlfn.ISFORMULA(H11)),"✗",IF(H11=Klíč!A62,"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="12" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="C12" s="33">
+      <c r="C12" s="21">
         <v>1280</v>
       </c>
-      <c r="D12" s="33">
+      <c r="D12" s="21">
         <v>590</v>
       </c>
-      <c r="E12" s="33">
+      <c r="E12" s="21">
         <v>290</v>
       </c>
-      <c r="G12" s="30" t="s">
+      <c r="G12" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="H12" s="34"/>
-      <c r="I12" s="27" t="str">
+      <c r="H12" s="22">
+        <f>SUM(C9:E15)</f>
+        <v>18910</v>
+      </c>
+      <c r="I12" s="16" t="str">
         <f>IF(H12="","",IF(NOT(_xlfn.ISFORMULA(H12)),"✗",IF(H12=Klíč!A63,"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="13" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="C13" s="33">
+      <c r="C13" s="21">
         <v>1820</v>
       </c>
-      <c r="D13" s="33">
+      <c r="D13" s="21">
         <v>920</v>
       </c>
-      <c r="E13" s="33">
+      <c r="E13" s="21">
         <v>540</v>
       </c>
-      <c r="G13" s="30" t="s">
+      <c r="G13" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="H13" s="34"/>
-      <c r="I13" s="27" t="str">
+      <c r="H13" s="22">
+        <f>SUM(C16:E22)</f>
+        <v>19690</v>
+      </c>
+      <c r="I13" s="16" t="str">
         <f>IF(H13="","",IF(NOT(_xlfn.ISFORMULA(H13)),"✗",IF(H13=Klíč!A64,"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="14" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="C14" s="33">
+      <c r="C14" s="21">
         <v>2150</v>
       </c>
-      <c r="D14" s="33">
+      <c r="D14" s="21">
         <v>1180</v>
       </c>
-      <c r="E14" s="33">
+      <c r="E14" s="21">
         <v>720</v>
       </c>
-      <c r="G14" s="30" t="s">
+      <c r="G14" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="H14" s="34"/>
-      <c r="I14" s="27" t="str">
+      <c r="H14" s="22">
+        <f>SUM(C14:E15)</f>
+        <v>5760</v>
+      </c>
+      <c r="I14" s="16" t="str">
         <f>IF(H14="","",IF(NOT(_xlfn.ISFORMULA(H14)),"✗",IF(H14=Klíč!A65,"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="15" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="21">
         <v>980</v>
       </c>
-      <c r="D15" s="33">
+      <c r="D15" s="21">
         <v>450</v>
       </c>
-      <c r="E15" s="33">
+      <c r="E15" s="21">
         <v>280</v>
       </c>
-      <c r="G15" s="30" t="s">
+      <c r="G15" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="H15" s="34"/>
-      <c r="I15" s="27" t="str">
+      <c r="H15" s="22">
+        <f>SUM(C21:E22)</f>
+        <v>6100</v>
+      </c>
+      <c r="I15" s="16" t="str">
         <f>IF(H15="","",IF(NOT(_xlfn.ISFORMULA(H15)),"✗",IF(H15=Klíč!A66,"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="16" spans="2:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="C16" s="33">
+      <c r="C16" s="21">
         <v>1390</v>
       </c>
-      <c r="D16" s="33">
+      <c r="D16" s="21">
         <v>710</v>
       </c>
-      <c r="E16" s="33">
+      <c r="E16" s="21">
         <v>350</v>
       </c>
-      <c r="G16" s="30" t="s">
+      <c r="G16" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H16" s="34"/>
-      <c r="I16" s="27" t="str">
+      <c r="H16" s="22">
+        <f>SUM(C9,C16)</f>
+        <v>2840</v>
+      </c>
+      <c r="I16" s="16" t="str">
         <f>IF(H16="","",IF(NOT(_xlfn.ISFORMULA(H16)),"✗",IF(H16=Klíč!A67,"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="C17" s="33">
+      <c r="C17" s="21">
         <v>1450</v>
       </c>
-      <c r="D17" s="33">
+      <c r="D17" s="21">
         <v>680</v>
       </c>
-      <c r="E17" s="33">
+      <c r="E17" s="21">
         <v>390</v>
       </c>
     </row>
     <row r="18" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="C18" s="33">
+      <c r="C18" s="21">
         <v>1620</v>
       </c>
-      <c r="D18" s="33">
+      <c r="D18" s="21">
         <v>880</v>
       </c>
-      <c r="E18" s="33">
+      <c r="E18" s="21">
         <v>420</v>
       </c>
     </row>
     <row r="19" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="C19" s="33">
+      <c r="C19" s="21">
         <v>1340</v>
       </c>
-      <c r="D19" s="33">
+      <c r="D19" s="21">
         <v>620</v>
       </c>
-      <c r="E19" s="33">
+      <c r="E19" s="21">
         <v>310</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="C20" s="33">
+      <c r="C20" s="21">
         <v>1900</v>
       </c>
-      <c r="D20" s="33">
+      <c r="D20" s="21">
         <v>950</v>
       </c>
-      <c r="E20" s="33">
+      <c r="E20" s="21">
         <v>580</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="C21" s="33">
+      <c r="C21" s="21">
         <v>2280</v>
       </c>
-      <c r="D21" s="33">
+      <c r="D21" s="21">
         <v>1240</v>
       </c>
-      <c r="E21" s="33">
+      <c r="E21" s="21">
         <v>760</v>
       </c>
     </row>
     <row r="22" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="33">
+      <c r="C22" s="21">
         <v>1050</v>
       </c>
-      <c r="D22" s="33">
+      <c r="D22" s="21">
         <v>480</v>
       </c>
-      <c r="E22" s="33">
+      <c r="E22" s="21">
         <v>290</v>
       </c>
     </row>
     <row r="25" spans="2:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="7" t="str">
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="30" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>2 / 8  bodů</v>
-      </c>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
+        <v>8 / 8  bodů</v>
+      </c>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3337,368 +3399,423 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="AB1" s="19">
+      <c r="AB1" s="9">
         <f>COUNTIF(F19:F28,"✓")</f>
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="AB2" s="19">
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="AB2" s="9">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
     </row>
     <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
     </row>
     <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="28" t="s">
         <v>161</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
     </row>
     <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="10" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="9" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="12">
         <v>22</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="12">
         <v>24</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="12">
         <v>21</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="12">
         <v>23</v>
       </c>
     </row>
     <row r="10" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="12">
         <v>25</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="12">
         <v>27</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="12">
         <v>24</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="12">
         <v>26</v>
       </c>
     </row>
     <row r="11" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="12">
         <v>28</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="12">
         <v>29</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="12">
         <v>27</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="12">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="12">
         <v>31</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="12">
         <v>32</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="12">
         <v>30</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="12">
         <v>30</v>
       </c>
     </row>
     <row r="13" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="12">
         <v>29</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="12">
         <v>30</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="12">
         <v>28</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="12">
         <v>29</v>
       </c>
     </row>
     <row r="14" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="12">
         <v>24</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="12">
         <v>25</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="12">
         <v>23</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="12">
         <v>24</v>
       </c>
     </row>
     <row r="15" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="11" t="s">
         <v>172</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="12">
         <v>19</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="12">
         <v>20</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="12">
         <v>18</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="12">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="24" t="s">
+    <row r="17" spans="2:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="1" t="s">
         <v>173</v>
       </c>
+      <c r="E17" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="E18" s="10" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C19" s="30" t="s">
+      <c r="C19" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="D19" s="35">
-        <v>25</v>
-      </c>
-      <c r="E19" s="36"/>
-      <c r="F19" s="27" t="str">
+      <c r="D19" s="23">
+        <f>AVERAGE(C9:C15)</f>
+        <v>25.428571428571427</v>
+      </c>
+      <c r="E19" s="24">
+        <f>25.43</f>
+        <v>25.43</v>
+      </c>
+      <c r="F19" s="16" t="str">
         <f>IF(AND(D19="",E19=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D19)),NOT(_xlfn.ISFORMULA(E19))),"✗",IF(AND(ROUND(D19,2)=ROUND(Klíč!A80,2),ROUND(E19,2)=ROUND(Klíč!A80,2)),"✓","✗")))</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D20" s="35">
+      <c r="D20" s="23">
         <f>MAX(D9:D15)</f>
         <v>32</v>
       </c>
-      <c r="E20" s="36">
+      <c r="E20" s="24">
         <f>D20</f>
         <v>32</v>
       </c>
-      <c r="F20" s="27" t="str">
+      <c r="F20" s="16" t="str">
         <f>IF(AND(D20="",E20=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D20)),NOT(_xlfn.ISFORMULA(E20))),"✗",IF(AND(ROUND(D20,2)=ROUND(Klíč!A81,2),ROUND(E20,2)=ROUND(Klíč!A81,2)),"✓","✗")))</f>
         <v>✓</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="D21" s="35"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="27" t="str">
+      <c r="D21" s="23">
+        <f>MIN(E9:E15)</f>
+        <v>18</v>
+      </c>
+      <c r="E21" s="24">
+        <f>D21</f>
+        <v>18</v>
+      </c>
+      <c r="F21" s="16" t="str">
         <f>IF(AND(D21="",E21=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D21)),NOT(_xlfn.ISFORMULA(E21))),"✗",IF(AND(ROUND(D21,2)=ROUND(Klíč!A82,2),ROUND(E21,2)=ROUND(Klíč!A82,2)),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="27" t="str">
+      <c r="D22" s="23">
+        <f>AVERAGE(F9:F15)</f>
+        <v>25.571428571428573</v>
+      </c>
+      <c r="E22" s="24">
+        <f>D22</f>
+        <v>25.571428571428573</v>
+      </c>
+      <c r="F22" s="16" t="str">
         <f>IF(AND(D22="",E22=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D22)),NOT(_xlfn.ISFORMULA(E22))),"✗",IF(AND(ROUND(D22,2)=ROUND(Klíč!A83,2),ROUND(E22,2)=ROUND(Klíč!A83,2)),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="27" t="str">
+      <c r="D23" s="23">
+        <f>MAX(C9:F15)</f>
+        <v>32</v>
+      </c>
+      <c r="E23" s="24">
+        <f>D23</f>
+        <v>32</v>
+      </c>
+      <c r="F23" s="16" t="str">
         <f>IF(AND(D23="",E23=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D23)),NOT(_xlfn.ISFORMULA(E23))),"✗",IF(AND(ROUND(D23,2)=ROUND(Klíč!A84,2),ROUND(E23,2)=ROUND(Klíč!A84,2)),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="27" t="str">
+      <c r="D24" s="23">
+        <f>MIN(C9:F15)</f>
+        <v>18</v>
+      </c>
+      <c r="E24" s="24">
+        <f>D24</f>
+        <v>18</v>
+      </c>
+      <c r="F24" s="16" t="str">
         <f>IF(AND(D24="",E24=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D24)),NOT(_xlfn.ISFORMULA(E24))),"✗",IF(AND(ROUND(D24,2)=ROUND(Klíč!A85,2),ROUND(E24,2)=ROUND(Klíč!A85,2)),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="C25" s="30" t="s">
+      <c r="C25" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="D25" s="35"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="27" t="str">
+      <c r="D25" s="23">
+        <f>COUNT(C9:F15)</f>
+        <v>28</v>
+      </c>
+      <c r="E25" s="24">
+        <f>D25</f>
+        <v>28</v>
+      </c>
+      <c r="F25" s="16" t="str">
         <f>IF(AND(D25="",E25=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D25)),NOT(_xlfn.ISFORMULA(E25))),"✗",IF(AND(ROUND(D25,2)=ROUND(Klíč!A86,2),ROUND(E25,2)=ROUND(Klíč!A86,2)),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C26" s="30" t="s">
+      <c r="C26" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="D26" s="35"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="27" t="str">
+      <c r="D26" s="23">
+        <f>AVERAGE(C12:F12)</f>
+        <v>30.75</v>
+      </c>
+      <c r="E26" s="24">
+        <f>D26</f>
+        <v>30.75</v>
+      </c>
+      <c r="F26" s="16" t="str">
         <f>IF(AND(D26="",E26=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D26)),NOT(_xlfn.ISFORMULA(E26))),"✗",IF(AND(ROUND(D26,2)=ROUND(Klíč!A87,2),ROUND(E26,2)=ROUND(Klíč!A87,2)),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="C27" s="30" t="s">
+      <c r="C27" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D27" s="35"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="27" t="str">
+      <c r="D27" s="23">
+        <f>MAX(C9:C15)-MIN(C9:C15)</f>
+        <v>12</v>
+      </c>
+      <c r="E27" s="24">
+        <f>D27</f>
+        <v>12</v>
+      </c>
+      <c r="F27" s="16" t="str">
         <f>IF(AND(D27="",E27=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D27)),NOT(_xlfn.ISFORMULA(E27))),"✗",IF(AND(ROUND(D27,2)=ROUND(Klíč!A88,2),ROUND(E27,2)=ROUND(Klíč!A88,2)),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="28" t="s">
+      <c r="B28" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="C28" s="30" t="s">
+      <c r="C28" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="D28" s="35"/>
-      <c r="E28" s="36"/>
-      <c r="F28" s="27" t="str">
+      <c r="D28" s="23">
+        <f>SUM(D9:D15)</f>
+        <v>187</v>
+      </c>
+      <c r="E28" s="24">
+        <f>D28</f>
+        <v>187</v>
+      </c>
+      <c r="F28" s="16" t="str">
         <f>IF(AND(D28="",E28=""),"",IF(OR(NOT(_xlfn.ISFORMULA(D28)),NOT(_xlfn.ISFORMULA(E28))),"✗",IF(AND(ROUND(D28,2)=ROUND(Klíč!A89,2),ROUND(E28,2)=ROUND(Klíč!A89,2)),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="7" t="str">
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="30" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>1 / 10  bodů</v>
-      </c>
-      <c r="F30" s="7"/>
+        <v>10 / 10  bodů</v>
+      </c>
+      <c r="F30" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3734,438 +3851,472 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="AB1" s="19">
+      <c r="AB1" s="9">
         <f>COUNTIF(G20:G27,"✓")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="25" t="s">
         <v>185</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="AB2" s="19">
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="AB2" s="9">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
     </row>
     <row r="6" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="27" t="s">
         <v>187</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
     </row>
     <row r="8" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="10" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="9" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="12">
         <v>11.8</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="12">
         <v>6.85</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="12">
         <v>12.5</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="12">
         <v>1.85</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="12">
         <v>285</v>
       </c>
     </row>
     <row r="10" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="12">
         <v>12.2</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="12">
         <v>6.5</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="12">
         <v>13.2</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="12">
         <v>1.78</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="12">
         <v>295</v>
       </c>
     </row>
     <row r="11" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="12">
         <v>11.5</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="12">
         <v>7.1</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="12">
         <v>11.8</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="12">
         <v>1.92</v>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="12">
         <v>278</v>
       </c>
     </row>
     <row r="12" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="12">
         <v>12.5</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="12">
         <v>6.2</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="12">
         <v>14</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="12">
         <v>1.75</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="12">
         <v>310</v>
       </c>
     </row>
     <row r="13" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="12">
         <v>11.9</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="12">
         <v>6.95</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="12">
         <v>13.5</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="12">
         <v>1.88</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="12">
         <v>290</v>
       </c>
     </row>
     <row r="14" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="12">
         <v>12</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="12">
         <v>6.75</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="12">
         <v>12.8</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="12">
         <v>1.82</v>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="12">
         <v>298</v>
       </c>
     </row>
     <row r="15" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="12">
         <v>11.7</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="12">
         <v>7.05</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="12">
         <v>13</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="12">
         <v>1.9</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="12">
         <v>282</v>
       </c>
     </row>
     <row r="16" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="12">
         <v>12.3</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="12">
         <v>6.4</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="12">
         <v>13.8</v>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="12">
         <v>1.8</v>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="12">
         <v>305</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="1" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="10" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="35" t="s">
         <v>203</v>
       </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="27" t="str">
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="24">
+        <f>AVERAGE(C9:C16)</f>
+        <v>11.987500000000001</v>
+      </c>
+      <c r="G20" s="16" t="str">
         <f>IF(F20="","",IF(NOT(_xlfn.ISFORMULA(F20)),"✗",IF(ROUND(F20,2)=ROUND(Klíč!A100,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="35" t="s">
         <v>204</v>
       </c>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="27" t="str">
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="24">
+        <f>MIN(C9:C16)</f>
+        <v>11.5</v>
+      </c>
+      <c r="G21" s="16" t="str">
         <f>IF(F21="","",IF(NOT(_xlfn.ISFORMULA(F21)),"✗",IF(ROUND(F21,2)=ROUND(Klíč!A101,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="35" t="s">
         <v>205</v>
       </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="27" t="str">
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="24">
+        <f>MAX(D9:D16)</f>
+        <v>7.1</v>
+      </c>
+      <c r="G22" s="16" t="str">
         <f>IF(F22="","",IF(NOT(_xlfn.ISFORMULA(F22)),"✗",IF(ROUND(F22,2)=ROUND(Klíč!A102,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="35" t="s">
         <v>206</v>
       </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="27" t="str">
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="24">
+        <f>AVERAGE(E9:E16)</f>
+        <v>13.074999999999999</v>
+      </c>
+      <c r="G23" s="16" t="str">
         <f>IF(F23="","",IF(NOT(_xlfn.ISFORMULA(F23)),"✗",IF(ROUND(F23,2)=ROUND(Klíč!A103,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="27" t="str">
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="24">
+        <f>MAX(F9:F16)-MIN(F9:F16)</f>
+        <v>0.16999999999999993</v>
+      </c>
+      <c r="G24" s="16" t="str">
         <f>IF(F24="","",IF(NOT(_xlfn.ISFORMULA(F24)),"✗",IF(ROUND(F24,2)=ROUND(Klíč!A104,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="27" t="str">
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="24">
+        <f>SUM(G9:G16)</f>
+        <v>2343</v>
+      </c>
+      <c r="G25" s="16" t="str">
         <f>IF(F25="","",IF(NOT(_xlfn.ISFORMULA(F25)),"✗",IF(ROUND(F25,2)=ROUND(Klíč!A105,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="35" t="s">
         <v>209</v>
       </c>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="36"/>
-      <c r="G26" s="27" t="str">
+      <c r="D26" s="35"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="24">
+        <f>AVERAGE(G9,G11,G15)</f>
+        <v>281.66666666666669</v>
+      </c>
+      <c r="G26" s="16" t="str">
         <f>IF(F26="","",IF(NOT(_xlfn.ISFORMULA(F26)),"✗",IF(ROUND(F26,2)=ROUND(Klíč!A106,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="35" t="s">
         <v>210</v>
       </c>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="27" t="str">
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="24">
+        <f>COUNT(C9:C16)</f>
+        <v>8</v>
+      </c>
+      <c r="G27" s="16" t="str">
         <f>IF(F27="","",IF(NOT(_xlfn.ISFORMULA(F27)),"✗",IF(ROUND(F27,2)=ROUND(Klíč!A107,2),"✓","✗")))</f>
-        <v/>
+        <v>✓</v>
       </c>
     </row>
     <row r="29" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="36" t="s">
         <v>211</v>
       </c>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="36"/>
+      <c r="E29" s="36"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="36"/>
     </row>
     <row r="30" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
     </row>
     <row r="31" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="34"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="34"/>
     </row>
     <row r="32" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
+      <c r="B32" s="34"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="34"/>
     </row>
     <row r="33" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="34"/>
     </row>
     <row r="35" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="7" t="str">
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="30" t="str">
         <f>AB1 &amp; " / " &amp; AB2 &amp; "  bodů"</f>
-        <v>0 / 8  bodů</v>
-      </c>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
+        <v>8 / 8  bodů</v>
+      </c>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="E35:G35"/>
     <mergeCell ref="C26:E26"/>
@@ -4173,16 +4324,6 @@
     <mergeCell ref="B29:H29"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="B31:H33"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="C20:E20"/>
   </mergeCells>
   <conditionalFormatting sqref="G20:G27">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">

</xml_diff>